<commit_message>
Update AI Audit Log Week 2
</commit_message>
<xml_diff>
--- a/SWR302_AI_Audit.xlsx
+++ b/SWR302_AI_Audit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_IT\Semester\SU26\SE20C02_LAB211_SU26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thuan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DB4BAFD-22E4-4A56-8BB6-7291655F4E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046D8E7E-F5D1-4F52-9BE4-60511859EE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -34,9 +34,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -44,27 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
-    <t>Ví dụ: Abstraction</t>
-  </si>
-  <si>
-    <t>“Tôi cần quản lý thông tin sinh viên cho app quản lý điểm. Hãy liệt kê các thuộc tính cần thiết."</t>
-  </si>
-  <si>
-    <t>Ví dụ: Process/Algorithm</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition</t>
-  </si>
-  <si>
-    <t>“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition + Literature Review</t>
-  </si>
-  <si>
-    <t>“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
-  </si>
-  <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
   <si>
@@ -77,23 +53,44 @@
     <t>STT</t>
   </si>
   <si>
-    <t>Phản hồi: AI liệt kê 20 thuộc tính.
-Quyết định: Tôi chỉ chọn 10 thuộc tính liên quan đến chức năng đang được yêu cầu từ ứng dụng (CCCD, địa chỉ...) và lược bỏ 10 thuộc tính học thuật vì phù hợp với yêu cầu của ứng dụng</t>
-  </si>
-  <si>
-    <t>"Viết hàm C sắp xếp mảng sinh viên theo điểm số bằng Selection Sort."</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI cung cấp code mẫu.
-Kiểm chứng: Tôi nhận thấy code AI chưa xử lý trường hợp mảng rỗng (Oversimplification). Tôi đã yêu cầu AI tối ưu lại và tự tay bổ sung điều kiện kiểm tra lỗi.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI response Round Robin là “tốt nhất” vì cân bằng giữa throughput và fairness.
-Kiểm chứng: AI đưa kết luận sai – không có giải thuật “tốt nhất” tuyệt đối (Hallucination). Mỗi giải thuật phù hợp với tình huống/context khác nhau.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI tóm tắt 5 papers với tên tác giả, năm xuất bản và tóm tắt nội dung.
-Kiểm chứng: Tìm trên Google Scholar: 2/5 papers AI nêu là không tồn tại (fabrication). Tôi đã thay bằng 2 papers mà tôi đã tìm kiếm trên research gates và đã kiểm chứng trên google scholar.</t>
+    <t>Actor Identification &amp; Security</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI gợi ý tạo một Actor User chung cho mọi đối tượng khách hàng, sau đó tạo một Use Case trung tâm là Login/Authenticate Account rồi dùng mũi tên &lt;&lt;include&gt;&gt; từ tất cả các Use Case nhạy cảm chỉ về nó.
+Kiểm chứng: Nếu dùng &lt;&lt;include&gt;&gt; từ mọi ô chức năng về phía Login, sơ đồ sẽ tràn ngập các đường mũi tên cắt chéo nhau (</t>
+  </si>
+  <si>
+    <t>Use Case Relationships</t>
+  </si>
+  <si>
+    <t>Để đặt chỗ, khách hàng phải trả trước trực tuyến. Cần thể hiện mối quan hệ này trên sơ đồ</t>
+  </si>
+  <si>
+    <t>Yêu cầu hệ thống đảm bảo chỉ những người dùng đã được xác thực mới có thể truy cập vào các thông tin nhạy cảm. Cần tìm phương án vẽ sạch sẽ, không rối dây.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI bị lỗi logic khi gợi ý vẽ mũi tên nét đứt &lt;&lt;include&gt;&gt; hướng trực tiếp từ hai Use Case công khai là Browse Space và Check Availability chỉ thẳng vào Make Payment
+Kiểm chứng: Sửa lại bằng cách giữ Browse Space và Check Availability đứng độc lập cho Guest xem thoải mái.</t>
+  </si>
+  <si>
+    <t>Use Case Relationships (Cancellation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiết lập mối quan hệ giữa chức năng Hủy đặt chỗ và Hoàn tiền </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phản hồi: AI hướng dẫn dùng mối quan hệ &lt;&lt;include&gt;&gt; chỉ từ Cancel Booking sang Refund Payment. Khi yêu cầu đổi sang &lt;&lt;Extend&gt;&gt;, AI lại hướng dẫn vẽ mũi tên nét đứt có đầu mũi tên chĩa từ Cancel Booking sang Refund.
+Kiểm chứng: đề bài ghi rõ: "Cancellations made 12 hours prior are refundable". Nghĩa là việc hoàn tiền chỉ là một nhánh mở rộng có điều kiện (tùy thuộc vào mốc thời gian), không phải cứ hủy lịch là mặc định được trả lại tiền --&gt; Phải dùng &lt;&lt;Extend&gt;&gt; chứ không được dùng &lt;&lt;Include&gt;&gt;. </t>
+  </si>
+  <si>
+    <t>Back-office Authentication &amp; Review</t>
+  </si>
+  <si>
+    <t>Sửa lại sơ đồ hiện rõ tính năng bảo mật đăng nhập cho cả Admin và Manager, đồng thời chuẩn hóa các tính năng duyệt chỗ trống của Admin mà không làm rối bố cục.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI gợi ý nhân bản (copy) Use Case Login Account ra thành 3-4 ô oval khác nhau đặt rải rác khắp nơi
+Kiểm chứng: Gom các chức năng duyệt vụn vặt (Review, Reject) của Admin thành một Use Case tổng quát là Approve Space Slots</t>
   </si>
 </sst>
 </file>
@@ -104,7 +101,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -113,7 +110,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -175,7 +172,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -508,80 +505,80 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBDDC7E-59F2-4CBB-B3D2-F6FB78F9E873}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.9296875" customWidth="1"/>
-    <col min="2" max="2" width="26.86328125" customWidth="1"/>
-    <col min="3" max="3" width="24.265625" customWidth="1"/>
+    <col min="1" max="1" width="20.9375" customWidth="1"/>
+    <col min="2" max="2" width="32.5625" customWidth="1"/>
+    <col min="3" max="3" width="24.25" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" ht="108" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" ht="94.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" ht="148.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="94.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>15</v>
@@ -595,7 +592,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E3EFE9-6FFB-49CC-BE69-0C0E36C6253E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -604,7 +601,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -613,7 +610,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>